<commit_message>
COMMIT 12 : upload des prix reste gestion du crash à terminer save-delete reload
</commit_message>
<xml_diff>
--- a/Sauvegarde/lastcash_2026-03-09.xlsx
+++ b/Sauvegarde/lastcash_2026-03-09.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -485,6 +485,32 @@
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Test2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>bp</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>